<commit_message>
Implemented simple headers, so the full path will not be shown as the header unless needed to differentiate it with other labels of the XML tree.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/project_task.xlsx
+++ b/project_task.xlsx
@@ -419,27 +419,27 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>task_task_id</t>
+          <t>task_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>task_project_name</t>
+          <t>project_name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>task_assigned_to</t>
+          <t>assigned_to</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>task_status</t>
+          <t>status</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>task_hours_logged</t>
+          <t>hours_logged</t>
         </is>
       </c>
     </row>

</xml_diff>